<commit_message>
new cases in excel file
</commit_message>
<xml_diff>
--- a/geothermal_surrogate_cases.xlsx
+++ b/geothermal_surrogate_cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\colli\OneDrive - JGU\13. Semester\running_geothermalwells.jl\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jgumainz-my.sharepoint.com/personal/cwittens_uni-mainz_de/Documents/13. Semester/running_geothermalwells.jl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B0E59BD-0EE2-4C5E-BA8C-E87CBA448A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{7B0E59BD-0EE2-4C5E-BA8C-E87CBA448A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99DFB100-935A-45F5-B3CF-A707084ECD83}"/>
   <bookViews>
-    <workbookView xWindow="4044" yWindow="17172" windowWidth="23256" windowHeight="12456" xr2:uid="{56B75647-DE6C-8F47-9018-5EF867A6E34A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{56B75647-DE6C-8F47-9018-5EF867A6E34A}"/>
   </bookViews>
   <sheets>
     <sheet name="geothermal_surrogate_cases" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="11">
   <si>
     <t>Case</t>
   </si>
@@ -59,7 +59,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -190,6 +190,12 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -548,10 +554,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -927,13 +934,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126A038D-7255-FB4F-8008-010C448053B0}">
-  <dimension ref="A1:J33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J48"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="10" max="10" width="103.375" customWidth="1"/>
+    <col min="10" max="10" width="103.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -960,7 +967,7 @@
       </c>
       <c r="J1" s="2"/>
     </row>
-    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -986,7 +993,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1012,7 +1019,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1038,7 +1045,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1064,7 +1071,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1090,7 +1097,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1116,7 +1123,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1142,7 +1149,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1168,7 +1175,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1194,7 +1201,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1220,7 +1227,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1246,7 +1253,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1272,7 +1279,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1298,7 +1305,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1324,7 +1331,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1350,7 +1357,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1376,7 +1383,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1402,7 +1409,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1428,7 +1435,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1454,7 +1461,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1480,7 +1487,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1506,7 +1513,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1532,7 +1539,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1558,7 +1565,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1584,7 +1591,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1610,7 +1617,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1636,7 +1643,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1662,7 +1669,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -1688,7 +1695,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -1714,7 +1721,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -1740,7 +1747,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -1766,7 +1773,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1792,7 +1799,346 @@
         <v>20</v>
       </c>
     </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>100</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D36" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E36" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F36" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G36" s="3">
+        <v>5</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>101</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D37" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E37" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F37" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G37" s="3">
+        <v>5</v>
+      </c>
+      <c r="H37" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>102</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D38" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E38" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F38" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G38" s="3">
+        <v>5</v>
+      </c>
+      <c r="H38" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
+        <v>103</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D39" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E39" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F39" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G39" s="3">
+        <v>5</v>
+      </c>
+      <c r="H39" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
+        <v>104</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D40" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E40" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F40" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G40" s="3">
+        <v>5</v>
+      </c>
+      <c r="H40" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
+        <v>105</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D41" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E41" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F41" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G41" s="3">
+        <v>5</v>
+      </c>
+      <c r="H41" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <v>106</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D42" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E42" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F42" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G42" s="3">
+        <v>5</v>
+      </c>
+      <c r="H42" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="3">
+        <v>107</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D43" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E43" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F43" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G43" s="3">
+        <v>5</v>
+      </c>
+      <c r="H43" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" s="3">
+        <v>108</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D44" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E44" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F44" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G44" s="3">
+        <v>5</v>
+      </c>
+      <c r="H44" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="3">
+        <v>109</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D45" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E45" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F45" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G45" s="3">
+        <v>5</v>
+      </c>
+      <c r="H45" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" s="3">
+        <v>110</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D46" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E46" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F46" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G46" s="3">
+        <v>5</v>
+      </c>
+      <c r="H46" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" s="3">
+        <v>111</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D47" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E47" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F47" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G47" s="3">
+        <v>5</v>
+      </c>
+      <c r="H47" s="3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48" s="3">
+        <v>112</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D48" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="E48" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F48" s="3">
+        <v>-400000</v>
+      </c>
+      <c r="G48" s="3">
+        <v>5</v>
+      </c>
+      <c r="H48" s="3">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new files with increasingly bigger spacing in the wells
</commit_message>
<xml_diff>
--- a/geothermal_surrogate_cases.xlsx
+++ b/geothermal_surrogate_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jgumainz-my.sharepoint.com/personal/cwittens_uni-mainz_de/Documents/13. Semester/running_geothermalwells.jl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{7B0E59BD-0EE2-4C5E-BA8C-E87CBA448A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99DFB100-935A-45F5-B3CF-A707084ECD83}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{7B0E59BD-0EE2-4C5E-BA8C-E87CBA448A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAD2D774-7082-4474-B932-9F018DD85D4D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{56B75647-DE6C-8F47-9018-5EF867A6E34A}"/>
+    <workbookView minimized="1" xWindow="5760" yWindow="2856" windowWidth="17280" windowHeight="8880" xr2:uid="{56B75647-DE6C-8F47-9018-5EF867A6E34A}"/>
   </bookViews>
   <sheets>
     <sheet name="geothermal_surrogate_cases" sheetId="1" r:id="rId1"/>
@@ -554,11 +554,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -615,6 +614,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1800,340 +1803,340 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="3">
+      <c r="A36">
         <v>100</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" t="s">
         <v>8</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C36">
         <v>2.8</v>
       </c>
-      <c r="D36" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E36" s="3">
+      <c r="D36">
+        <v>2000000</v>
+      </c>
+      <c r="E36">
         <v>2000</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F36">
         <v>-400000</v>
       </c>
-      <c r="G36" s="3">
-        <v>5</v>
-      </c>
-      <c r="H36" s="3" t="s">
+      <c r="G36">
+        <v>5</v>
+      </c>
+      <c r="H36" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="3">
+      <c r="A37">
         <v>101</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" s="3">
+      <c r="B37" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37">
         <v>2.8</v>
       </c>
-      <c r="D37" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E37" s="3">
+      <c r="D37">
+        <v>2000000</v>
+      </c>
+      <c r="E37">
         <v>2000</v>
       </c>
-      <c r="F37" s="3">
+      <c r="F37">
         <v>-400000</v>
       </c>
-      <c r="G37" s="3">
-        <v>5</v>
-      </c>
-      <c r="H37" s="3">
+      <c r="G37">
+        <v>5</v>
+      </c>
+      <c r="H37">
         <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="3">
+      <c r="A38">
         <v>102</v>
       </c>
-      <c r="B38" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C38" s="3">
+      <c r="B38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38">
         <v>2.8</v>
       </c>
-      <c r="D38" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E38" s="3">
+      <c r="D38">
+        <v>2000000</v>
+      </c>
+      <c r="E38">
         <v>2000</v>
       </c>
-      <c r="F38" s="3">
+      <c r="F38">
         <v>-400000</v>
       </c>
-      <c r="G38" s="3">
-        <v>5</v>
-      </c>
-      <c r="H38" s="3">
+      <c r="G38">
+        <v>5</v>
+      </c>
+      <c r="H38">
         <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="3">
+      <c r="A39">
         <v>103</v>
       </c>
-      <c r="B39" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C39" s="3">
+      <c r="B39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39">
         <v>2.8</v>
       </c>
-      <c r="D39" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E39" s="3">
+      <c r="D39">
+        <v>2000000</v>
+      </c>
+      <c r="E39">
         <v>2000</v>
       </c>
-      <c r="F39" s="3">
+      <c r="F39">
         <v>-400000</v>
       </c>
-      <c r="G39" s="3">
-        <v>5</v>
-      </c>
-      <c r="H39" s="3">
+      <c r="G39">
+        <v>5</v>
+      </c>
+      <c r="H39">
         <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="3">
+      <c r="A40">
         <v>104</v>
       </c>
-      <c r="B40" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C40" s="3">
+      <c r="B40" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40">
         <v>2.8</v>
       </c>
-      <c r="D40" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E40" s="3">
+      <c r="D40">
+        <v>2000000</v>
+      </c>
+      <c r="E40">
         <v>2000</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40">
         <v>-400000</v>
       </c>
-      <c r="G40" s="3">
-        <v>5</v>
-      </c>
-      <c r="H40" s="3">
+      <c r="G40">
+        <v>5</v>
+      </c>
+      <c r="H40">
         <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" s="3">
+      <c r="A41">
         <v>105</v>
       </c>
-      <c r="B41" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C41" s="3">
+      <c r="B41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41">
         <v>2.8</v>
       </c>
-      <c r="D41" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E41" s="3">
+      <c r="D41">
+        <v>2000000</v>
+      </c>
+      <c r="E41">
         <v>2000</v>
       </c>
-      <c r="F41" s="3">
+      <c r="F41">
         <v>-400000</v>
       </c>
-      <c r="G41" s="3">
-        <v>5</v>
-      </c>
-      <c r="H41" s="3">
+      <c r="G41">
+        <v>5</v>
+      </c>
+      <c r="H41">
         <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42" s="3">
+      <c r="A42">
         <v>106</v>
       </c>
-      <c r="B42" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C42" s="3">
+      <c r="B42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42">
         <v>2.8</v>
       </c>
-      <c r="D42" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E42" s="3">
+      <c r="D42">
+        <v>2000000</v>
+      </c>
+      <c r="E42">
         <v>2000</v>
       </c>
-      <c r="F42" s="3">
+      <c r="F42">
         <v>-400000</v>
       </c>
-      <c r="G42" s="3">
-        <v>5</v>
-      </c>
-      <c r="H42" s="3">
+      <c r="G42">
+        <v>5</v>
+      </c>
+      <c r="H42">
         <v>60</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" s="3">
+      <c r="A43">
         <v>107</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" s="3">
+      <c r="B43" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43">
         <v>2.8</v>
       </c>
-      <c r="D43" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E43" s="3">
+      <c r="D43">
+        <v>2000000</v>
+      </c>
+      <c r="E43">
         <v>2000</v>
       </c>
-      <c r="F43" s="3">
+      <c r="F43">
         <v>-400000</v>
       </c>
-      <c r="G43" s="3">
-        <v>5</v>
-      </c>
-      <c r="H43" s="3">
+      <c r="G43">
+        <v>5</v>
+      </c>
+      <c r="H43">
         <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="3">
+      <c r="A44">
         <v>108</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" s="3">
+      <c r="B44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44">
         <v>2.8</v>
       </c>
-      <c r="D44" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E44" s="3">
+      <c r="D44">
+        <v>2000000</v>
+      </c>
+      <c r="E44">
         <v>2000</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F44">
         <v>-400000</v>
       </c>
-      <c r="G44" s="3">
-        <v>5</v>
-      </c>
-      <c r="H44" s="3">
+      <c r="G44">
+        <v>5</v>
+      </c>
+      <c r="H44">
         <v>80</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="3">
+      <c r="A45">
         <v>109</v>
       </c>
-      <c r="B45" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" s="3">
+      <c r="B45" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45">
         <v>2.8</v>
       </c>
-      <c r="D45" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E45" s="3">
+      <c r="D45">
+        <v>2000000</v>
+      </c>
+      <c r="E45">
         <v>2000</v>
       </c>
-      <c r="F45" s="3">
+      <c r="F45">
         <v>-400000</v>
       </c>
-      <c r="G45" s="3">
-        <v>5</v>
-      </c>
-      <c r="H45" s="3">
+      <c r="G45">
+        <v>5</v>
+      </c>
+      <c r="H45">
         <v>90</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="3">
+      <c r="A46">
         <v>110</v>
       </c>
-      <c r="B46" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" s="3">
+      <c r="B46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46">
         <v>2.8</v>
       </c>
-      <c r="D46" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E46" s="3">
+      <c r="D46">
+        <v>2000000</v>
+      </c>
+      <c r="E46">
         <v>2000</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46">
         <v>-400000</v>
       </c>
-      <c r="G46" s="3">
-        <v>5</v>
-      </c>
-      <c r="H46" s="3">
+      <c r="G46">
+        <v>5</v>
+      </c>
+      <c r="H46">
         <v>100</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A47" s="3">
+      <c r="A47">
         <v>111</v>
       </c>
-      <c r="B47" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C47" s="3">
+      <c r="B47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47">
         <v>2.8</v>
       </c>
-      <c r="D47" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E47" s="3">
+      <c r="D47">
+        <v>2000000</v>
+      </c>
+      <c r="E47">
         <v>2000</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F47">
         <v>-400000</v>
       </c>
-      <c r="G47" s="3">
-        <v>5</v>
-      </c>
-      <c r="H47" s="3">
+      <c r="G47">
+        <v>5</v>
+      </c>
+      <c r="H47">
         <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A48" s="3">
+      <c r="A48">
         <v>112</v>
       </c>
-      <c r="B48" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C48" s="3">
+      <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48">
         <v>2.8</v>
       </c>
-      <c r="D48" s="3">
-        <v>2000000</v>
-      </c>
-      <c r="E48" s="3">
+      <c r="D48">
+        <v>2000000</v>
+      </c>
+      <c r="E48">
         <v>2000</v>
       </c>
-      <c r="F48" s="3">
+      <c r="F48">
         <v>-400000</v>
       </c>
-      <c r="G48" s="3">
-        <v>5</v>
-      </c>
-      <c r="H48" s="3">
+      <c r="G48">
+        <v>5</v>
+      </c>
+      <c r="H48">
         <v>120</v>
       </c>
     </row>

</xml_diff>